<commit_message>
JLCPCB: expand designator ranges so BOM matches CPL
JLC's "BOM doesn't match CPL" was caused by KiCad-style ranges in the BOM
Designator field (e.g. "C12-C15", "D1-D6", "Q16-Q27") -- JLC read each range
as one literal designator that had no counterpart in the per-part CPL.

Expand every range to explicit comma-separated designators in the BOM (and the
THT reference). Verified: 177 BOM designator instances == 177 CPL designators,
unique 177 each, zero duplicates, zero set differences. Use the .csv files
(the hand-rolled .xlsx trips JLC's stricter server-side parser).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pcb/fab_release/jlcpcb/BOM_JLC-assembly.xlsx
+++ b/pcb/fab_release/jlcpcb/BOM_JLC-assembly.xlsx
@@ -84,7 +84,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">C2,C3,C6,C8,C12-C15,C19,C20,C23</t>
+          <t xml:space="preserve">C2,C3,C6,C8,C12,C13,C14,C15,C19,C20,C23</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -216,7 +216,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">D1-D6</t>
+          <t xml:space="preserve">D1,D2,D3,D4,D5,D6</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -238,7 +238,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">D15-D22</t>
+          <t xml:space="preserve">D15,D16,D17,D18,D19,D20,D21,D22</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -260,7 +260,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">D23-D28</t>
+          <t xml:space="preserve">D23,D24,D25,D26,D27,D28</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -502,7 +502,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">LS1-LS8</t>
+          <t xml:space="preserve">LS1,LS2,LS3,LS4,LS5,LS6,LS7,LS8</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -546,7 +546,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q2-Q7</t>
+          <t xml:space="preserve">Q2,Q3,Q4,Q5,Q6,Q7</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -568,7 +568,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q16-Q27</t>
+          <t xml:space="preserve">Q16,Q17,Q18,Q19,Q20,Q21,Q22,Q23,Q24,Q25,Q26,Q27</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -590,7 +590,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q28-Q33</t>
+          <t xml:space="preserve">Q28,Q29,Q30,Q31,Q32,Q33</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -634,7 +634,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">R1,R2,R61-R64,R69,R73,R75,R76</t>
+          <t xml:space="preserve">R1,R2,R61,R62,R63,R64,R69,R73,R75,R76</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -678,7 +678,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">R6-R11,R55,R65,R67,R79,R80</t>
+          <t xml:space="preserve">R6,R7,R8,R9,R10,R11,R55,R65,R67,R79,R80</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -788,7 +788,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">R41-R54,R57,R58</t>
+          <t xml:space="preserve">R41,R42,R43,R44,R45,R46,R47,R48,R49,R50,R51,R52,R53,R54,R57,R58</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">

</xml_diff>

<commit_message>
JLCPCB: resolve stock shortage -- revert 100k/22uF-1210 to exact design parts
JLC's parts review flagged 8 lines as assembly-stock short. Fixes:
- 100k 0805: C17407 (Basic, short) -> C96346 (Yageo RC0805FR-07100KL, the exact
  design part, in stock).
- 22uF/25V 1210: C307586 (short) -> C52306 (Samsung CL32A226KAJNNNE, the exact
  design part, in stock).
- U1 (AP63203 buck), BZ1 (buzzer), SW1-4 (tact) have no safe footprint/pinout
  drop-in; ORDERING documents reduce-qty / pre-order / DNP+hand-solder instead.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pcb/fab_release/jlcpcb/BOM_JLC-assembly.xlsx
+++ b/pcb/fab_release/jlcpcb/BOM_JLC-assembly.xlsx
@@ -182,7 +182,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">C307586</t>
+          <t xml:space="preserve">C52306</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t xml:space="preserve">C17407</t>
+          <t xml:space="preserve">C96346</t>
         </is>
       </c>
     </row>

</xml_diff>